<commit_message>
change head table dataset excel
</commit_message>
<xml_diff>
--- a/data collecting.xlsx
+++ b/data collecting.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phure\เอกสาร\GitHub\c-sorting-algorithm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280E8795-C449-4911-9272-6FED896CBA1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC2BEA8A-73BA-4406-858C-BC6468555658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{D32EC7AF-07E4-482F-A8FA-A097486C4469}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D32EC7AF-07E4-482F-A8FA-A097486C4469}"/>
   </bookViews>
   <sheets>
     <sheet name="Random" sheetId="1" r:id="rId1"/>
@@ -305,18 +305,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -467,22 +467,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -580,22 +580,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1130,22 +1130,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1243,22 +1243,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1793,22 +1793,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1906,22 +1906,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2456,22 +2456,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2569,22 +2569,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3119,22 +3119,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3232,22 +3232,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3822,22 +3822,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3913,22 +3913,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4008,22 +4008,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4099,22 +4099,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4192,22 +4192,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4282,22 +4282,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4351,7 +4351,7 @@
         <c:axId val="684990623"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="50000"/>
+          <c:max val="200000"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -4463,7 +4463,6 @@
         <c:crossAx val="685575535"/>
         <c:crossesAt val="1.0000000000000002E-3"/>
         <c:crossBetween val="midCat"/>
-        <c:majorUnit val="5000"/>
       </c:valAx>
       <c:valAx>
         <c:axId val="685575535"/>
@@ -4560,7 +4559,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0000" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="cross"/>
         <c:minorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
@@ -4801,22 +4800,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4914,22 +4913,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5464,22 +5463,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5577,22 +5576,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6127,22 +6126,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6240,22 +6239,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6790,22 +6789,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6903,22 +6902,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7453,22 +7452,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7566,22 +7565,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8116,22 +8115,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8229,22 +8228,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8771,22 +8770,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8884,22 +8883,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9461,22 +9460,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9552,22 +9551,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9647,22 +9646,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9738,22 +9737,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9831,22 +9830,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9921,22 +9920,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9990,7 +9989,7 @@
         <c:axId val="684990623"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="50000"/>
+          <c:max val="200000"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -10102,7 +10101,6 @@
         <c:crossAx val="685575535"/>
         <c:crossesAt val="1.0000000000000002E-3"/>
         <c:crossBetween val="midCat"/>
-        <c:majorUnit val="5000"/>
       </c:valAx>
       <c:valAx>
         <c:axId val="685575535"/>
@@ -10199,7 +10197,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0000" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="cross"/>
         <c:minorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
@@ -10440,22 +10438,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10553,22 +10551,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11103,22 +11101,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11216,22 +11214,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11766,22 +11764,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11879,22 +11877,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12429,22 +12427,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12542,22 +12540,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13148,22 +13146,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13239,22 +13237,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13334,22 +13332,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13425,22 +13423,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13518,22 +13516,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13608,22 +13606,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13677,7 +13675,7 @@
         <c:axId val="684990623"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="50000"/>
+          <c:max val="200000"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -13797,7 +13795,6 @@
         <c:crossAx val="685575535"/>
         <c:crossesAt val="1.0000000000000002E-3"/>
         <c:crossBetween val="midCat"/>
-        <c:majorUnit val="5000"/>
       </c:valAx>
       <c:valAx>
         <c:axId val="685575535"/>
@@ -13894,7 +13891,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0000" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="cross"/>
         <c:minorTickMark val="in"/>
         <c:tickLblPos val="nextTo"/>
@@ -14135,22 +14132,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -14248,22 +14245,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -14790,22 +14787,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -14903,22 +14900,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>500</c:v>
+                  <c:v>5000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1000</c:v>
+                  <c:v>10000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5000</c:v>
+                  <c:v>50000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -28154,10 +28151,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
+      <c r="B1" s="18"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
@@ -28165,21 +28162,21 @@
       </c>
       <c r="C3" s="1">
         <f>C35</f>
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="N3" s="4" t="s">
         <v>12</v>
       </c>
       <c r="O3" s="1">
         <f>D35</f>
-        <v>500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="16" t="s">
         <v>15</v>
       </c>
       <c r="D4" s="14"/>
@@ -28194,7 +28191,7 @@
       <c r="N4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="O4" s="16" t="s">
         <v>15</v>
       </c>
       <c r="P4" s="14"/>
@@ -28685,21 +28682,21 @@
       </c>
       <c r="C13" s="1">
         <f>E35</f>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="N13" s="4" t="s">
         <v>12</v>
       </c>
       <c r="O13" s="1">
         <f>F35</f>
-        <v>5000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="16" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="14"/>
@@ -28714,7 +28711,7 @@
       <c r="N14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="O14" s="13" t="s">
+      <c r="O14" s="16" t="s">
         <v>15</v>
       </c>
       <c r="P14" s="14"/>
@@ -29205,21 +29202,21 @@
       </c>
       <c r="C23" s="1">
         <f>G35</f>
-        <v>10000</v>
+        <v>100000</v>
       </c>
       <c r="N23" s="4" t="s">
         <v>12</v>
       </c>
       <c r="O23" s="1">
         <f>H35</f>
-        <v>50000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="24" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B24" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="16" t="s">
         <v>15</v>
       </c>
       <c r="D24" s="14"/>
@@ -29234,7 +29231,7 @@
       <c r="N24" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="O24" s="13" t="s">
+      <c r="O24" s="16" t="s">
         <v>15</v>
       </c>
       <c r="P24" s="14"/>
@@ -29723,7 +29720,7 @@
       <c r="B34" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C34" s="18" t="s">
+      <c r="C34" s="13" t="s">
         <v>22</v>
       </c>
       <c r="D34" s="14"/>
@@ -29756,22 +29753,22 @@
     <row r="35" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B35" s="12"/>
       <c r="C35" s="2">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="D35" s="2">
-        <v>500</v>
+        <v>5000</v>
       </c>
       <c r="E35" s="2">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="F35" s="2">
-        <v>5000</v>
+        <v>50000</v>
       </c>
       <c r="G35" s="2">
-        <v>10000</v>
+        <v>100000</v>
       </c>
       <c r="H35" s="2">
-        <v>50000</v>
+        <v>200000</v>
       </c>
       <c r="K35" s="1" t="s">
         <v>27</v>
@@ -30040,10 +30037,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="17"/>
+      <c r="B1" s="18"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
@@ -30051,21 +30048,21 @@
       </c>
       <c r="C3" s="1">
         <f>C35</f>
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="N3" s="4" t="s">
         <v>12</v>
       </c>
       <c r="O3" s="1">
         <f>D35</f>
-        <v>500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="16" t="s">
         <v>15</v>
       </c>
       <c r="D4" s="14"/>
@@ -30080,7 +30077,7 @@
       <c r="N4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="O4" s="16" t="s">
         <v>15</v>
       </c>
       <c r="P4" s="14"/>
@@ -30571,21 +30568,21 @@
       </c>
       <c r="C13" s="1">
         <f>E35</f>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="N13" s="4" t="s">
         <v>12</v>
       </c>
       <c r="O13" s="1">
         <f>F35</f>
-        <v>5000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="16" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="14"/>
@@ -30600,7 +30597,7 @@
       <c r="N14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="O14" s="13" t="s">
+      <c r="O14" s="16" t="s">
         <v>15</v>
       </c>
       <c r="P14" s="14"/>
@@ -31091,21 +31088,21 @@
       </c>
       <c r="C23" s="1">
         <f>G35</f>
-        <v>10000</v>
+        <v>100000</v>
       </c>
       <c r="N23" s="4" t="s">
         <v>12</v>
       </c>
       <c r="O23" s="1">
         <f>H35</f>
-        <v>50000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="24" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B24" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="16" t="s">
         <v>15</v>
       </c>
       <c r="D24" s="14"/>
@@ -31120,7 +31117,7 @@
       <c r="N24" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="O24" s="13" t="s">
+      <c r="O24" s="16" t="s">
         <v>15</v>
       </c>
       <c r="P24" s="14"/>
@@ -31609,7 +31606,7 @@
       <c r="B34" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C34" s="18" t="s">
+      <c r="C34" s="13" t="s">
         <v>22</v>
       </c>
       <c r="D34" s="14"/>
@@ -31642,22 +31639,22 @@
     <row r="35" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B35" s="12"/>
       <c r="C35" s="2">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="D35" s="2">
-        <v>500</v>
+        <v>5000</v>
       </c>
       <c r="E35" s="2">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="F35" s="2">
-        <v>5000</v>
+        <v>50000</v>
       </c>
       <c r="G35" s="2">
-        <v>10000</v>
+        <v>100000</v>
       </c>
       <c r="H35" s="2">
-        <v>50000</v>
+        <v>200000</v>
       </c>
       <c r="K35" s="1" t="s">
         <v>27</v>
@@ -31886,11 +31883,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:L24"/>
-    <mergeCell ref="N24:N25"/>
     <mergeCell ref="O24:X24"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="B4:B5"/>
@@ -31901,6 +31893,11 @@
     <mergeCell ref="C14:L14"/>
     <mergeCell ref="N14:N15"/>
     <mergeCell ref="O14:X14"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:L24"/>
+    <mergeCell ref="N24:N25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -31923,10 +31920,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="17"/>
+      <c r="B1" s="18"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
@@ -31934,21 +31931,21 @@
       </c>
       <c r="C3" s="1">
         <f>C35</f>
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="N3" s="4" t="s">
         <v>12</v>
       </c>
       <c r="O3" s="1">
         <f>D35</f>
-        <v>500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="16" t="s">
         <v>15</v>
       </c>
       <c r="D4" s="14"/>
@@ -31963,7 +31960,7 @@
       <c r="N4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="O4" s="16" t="s">
         <v>15</v>
       </c>
       <c r="P4" s="14"/>
@@ -32454,21 +32451,21 @@
       </c>
       <c r="C13" s="1">
         <f>E35</f>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="N13" s="4" t="s">
         <v>12</v>
       </c>
       <c r="O13" s="1">
         <f>F35</f>
-        <v>5000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="16" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="14"/>
@@ -32483,7 +32480,7 @@
       <c r="N14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="O14" s="13" t="s">
+      <c r="O14" s="16" t="s">
         <v>15</v>
       </c>
       <c r="P14" s="14"/>
@@ -32974,21 +32971,21 @@
       </c>
       <c r="C23" s="1">
         <f>G35</f>
-        <v>10000</v>
+        <v>100000</v>
       </c>
       <c r="N23" s="4" t="s">
         <v>12</v>
       </c>
       <c r="O23" s="1">
         <f>H35</f>
-        <v>50000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="24" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B24" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="16" t="s">
         <v>15</v>
       </c>
       <c r="D24" s="14"/>
@@ -33003,7 +33000,7 @@
       <c r="N24" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="O24" s="13" t="s">
+      <c r="O24" s="16" t="s">
         <v>15</v>
       </c>
       <c r="P24" s="14"/>
@@ -33492,7 +33489,7 @@
       <c r="B34" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C34" s="18" t="s">
+      <c r="C34" s="13" t="s">
         <v>22</v>
       </c>
       <c r="D34" s="14"/>
@@ -33525,22 +33522,22 @@
     <row r="35" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B35" s="12"/>
       <c r="C35" s="2">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="D35" s="2">
-        <v>500</v>
+        <v>5000</v>
       </c>
       <c r="E35" s="2">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="F35" s="2">
-        <v>5000</v>
+        <v>50000</v>
       </c>
       <c r="G35" s="2">
-        <v>10000</v>
+        <v>100000</v>
       </c>
       <c r="H35" s="2">
-        <v>50000</v>
+        <v>200000</v>
       </c>
       <c r="K35" s="1" t="s">
         <v>27</v>
@@ -33769,11 +33766,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:L24"/>
-    <mergeCell ref="N24:N25"/>
     <mergeCell ref="O24:X24"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="B4:B5"/>
@@ -33784,6 +33776,11 @@
     <mergeCell ref="C14:L14"/>
     <mergeCell ref="N14:N15"/>
     <mergeCell ref="O14:X14"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:L24"/>
+    <mergeCell ref="N24:N25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>